<commit_message>
description ar and en
</commit_message>
<xml_diff>
--- a/product_upload/packages/10/file.xlsx
+++ b/product_upload/packages/10/file.xlsx
@@ -1084,8 +1084,16 @@
           <t>6164034851-145-492213171976</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>وصف تفصيلي لـ XANAX 1 MG TABLET</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>XANAX 1 MG TABLET detailed description.</t>
+        </is>
+      </c>
       <c r="I4" t="n">
         <v>0</v>
       </c>
@@ -2067,8 +2075,16 @@
           <t>7865810267-230-187799395811</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>وصف تفصيلي لـ RIVOTRIL TAB 2 MG</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>RIVOTRIL TAB 2 MG detailed description.</t>
+        </is>
+      </c>
       <c r="I9" t="n">
         <v>0</v>
       </c>
@@ -2859,8 +2875,16 @@
           <t>3864745957-718-920620555014</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>وصف تفصيلي لـ RISPERDAL 4MG TAB</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>RISPERDAL 4MG TAB detailed description.</t>
+        </is>
+      </c>
       <c r="I13" t="inlineStr">
         <is>
           <t>SAJA-SAUDI ARABIAN JAPANESE PHARMACEUTICAL CO</t>
@@ -3048,8 +3072,16 @@
           <t>3563257332-993-855667034970</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>وصف تفصيلي لـ ROBITUSSIN-PE SYRUP</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>ROBITUSSIN-PE SYRUP detailed description.</t>
+        </is>
+      </c>
       <c r="I14" t="n">
         <v>0</v>
       </c>
@@ -3625,8 +3657,16 @@
           <t>4991499352-808-631317773731</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>وصف تفصيلي لـ ROFENAC GEL 1%</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>ROFENAC GEL 1% detailed description.</t>
+        </is>
+      </c>
       <c r="I17" t="n">
         <v>0</v>
       </c>
@@ -4007,8 +4047,16 @@
           <t>2037918799-335-295950685973</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>وصف تفصيلي لـ RISPERDAL 3MG TAB</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>RISPERDAL 3MG TAB detailed description.</t>
+        </is>
+      </c>
       <c r="I19" t="inlineStr">
         <is>
           <t>SAJA-SAUDI ARABIAN JAPANESE PHARMACEUTICAL CO</t>
@@ -4586,8 +4634,16 @@
           <t>6002858565-318-639135647149</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr"/>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>وصف تفصيلي لـ ROFENAC 100 MG SUPP</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>ROFENAC 100 MG SUPP detailed description.</t>
+        </is>
+      </c>
       <c r="I22" t="n">
         <v>0</v>
       </c>
@@ -4968,8 +5024,16 @@
           <t>7316023852-101-829367956420</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr"/>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>وصف تفصيلي لـ RISPERDAL 2MG TAB</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>RISPERDAL 2MG TAB detailed description.</t>
+        </is>
+      </c>
       <c r="I24" t="inlineStr">
         <is>
           <t>SAJA-SAUDI ARABIAN JAPANESE PHARMACEUTICAL CO</t>
@@ -5161,8 +5225,16 @@
           <t>2003319794-712-146043746999</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr"/>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>وصف تفصيلي لـ RINGERS INJECATION 500 ML SOLUTION</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>RINGERS INJECATION 500 ML SOLUTION detailed description.</t>
+        </is>
+      </c>
       <c r="I25" t="n">
         <v>0</v>
       </c>
@@ -5356,8 +5428,16 @@
           <t>0625919728-222-575006165263</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr"/>
-      <c r="H26" t="inlineStr"/>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>وصف تفصيلي لـ RINGER SOLUTION I.V INFUSION</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>RINGER SOLUTION I.V INFUSION detailed description.</t>
+        </is>
+      </c>
       <c r="I26" t="n">
         <v>0</v>
       </c>
@@ -5543,8 +5623,16 @@
           <t>3657242743-800-004851223244</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr"/>
-      <c r="H27" t="inlineStr"/>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>وصف تفصيلي لـ RIMACTANE 300 MG CAP</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>RIMACTANE 300 MG CAP detailed description.</t>
+        </is>
+      </c>
       <c r="I27" t="n">
         <v>0</v>
       </c>
@@ -5734,8 +5822,16 @@
           <t>5229329175-699-447242275477</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr"/>
-      <c r="H28" t="inlineStr"/>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>وصف تفصيلي لـ RIMACTANE  150 MG CAP</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>RIMACTANE  150 MG CAP detailed description.</t>
+        </is>
+      </c>
       <c r="I28" t="n">
         <v>0</v>
       </c>
@@ -6331,8 +6427,16 @@
           <t>6307509502-061-192959502102</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr"/>
-      <c r="H31" t="inlineStr"/>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>وصف تفصيلي لـ RINGERS SOLUTION</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>RINGERS SOLUTION detailed description.</t>
+        </is>
+      </c>
       <c r="I31" t="n">
         <v>0</v>
       </c>
@@ -6522,8 +6626,16 @@
           <t>0183508436-471-473635255993</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr"/>
-      <c r="H32" t="inlineStr"/>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>وصف تفصيلي لـ RINGERS SOLUTION</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>RINGERS SOLUTION detailed description.</t>
+        </is>
+      </c>
       <c r="I32" t="n">
         <v>0</v>
       </c>
@@ -6902,8 +7014,16 @@
           <t>0529653529-071-439539676499</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr"/>
-      <c r="H34" t="inlineStr"/>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>وصف تفصيلي لـ RISPERDAL 1MG TAB</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>RISPERDAL 1MG TAB detailed description.</t>
+        </is>
+      </c>
       <c r="I34" t="n">
         <v>0</v>
       </c>
@@ -7089,8 +7209,16 @@
           <t>9827710049-086-223082352714</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr"/>
-      <c r="H35" t="inlineStr"/>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>وصف تفصيلي لـ RISIDONE 1MG/1ML ORAL SOLUTION</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>RISIDONE 1MG/1ML ORAL SOLUTION detailed description.</t>
+        </is>
+      </c>
       <c r="I35" t="n">
         <v>0</v>
       </c>
@@ -8068,8 +8196,16 @@
           <t>5098771680-994-700602742789</t>
         </is>
       </c>
-      <c r="G40" t="inlineStr"/>
-      <c r="H40" t="inlineStr"/>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>وصف تفصيلي لـ RISPERDAL 2MG TAB</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>RISPERDAL 2MG TAB detailed description.</t>
+        </is>
+      </c>
       <c r="I40" t="inlineStr">
         <is>
           <t>SAJA-SAUDI ARABIAN JAPANESE PHARMACEUTICAL CO</t>
@@ -8647,8 +8783,16 @@
           <t>3590509595-659-851932339520</t>
         </is>
       </c>
-      <c r="G43" t="inlineStr"/>
-      <c r="H43" t="inlineStr"/>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>وصف تفصيلي لـ RINGERS SOLUTION</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>RINGERS SOLUTION detailed description.</t>
+        </is>
+      </c>
       <c r="I43" t="n">
         <v>0</v>
       </c>
@@ -8838,8 +8982,16 @@
           <t>5579557505-697-823838176510</t>
         </is>
       </c>
-      <c r="G44" t="inlineStr"/>
-      <c r="H44" t="inlineStr"/>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>وصف تفصيلي لـ RINGERS SOLUTION</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>RINGERS SOLUTION detailed description.</t>
+        </is>
+      </c>
       <c r="I44" t="n">
         <v>0</v>
       </c>
@@ -9029,8 +9181,16 @@
           <t>8412433803-850-111465490765</t>
         </is>
       </c>
-      <c r="G45" t="inlineStr"/>
-      <c r="H45" t="inlineStr"/>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>وصف تفصيلي لـ RINGERS SOLUTION</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>RINGERS SOLUTION detailed description.</t>
+        </is>
+      </c>
       <c r="I45" t="n">
         <v>0</v>
       </c>
@@ -9216,8 +9376,16 @@
           <t>9693560533-200-022670724902</t>
         </is>
       </c>
-      <c r="G46" t="inlineStr"/>
-      <c r="H46" t="inlineStr"/>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>وصف تفصيلي لـ RINGERS SOLUTION</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>RINGERS SOLUTION detailed description.</t>
+        </is>
+      </c>
       <c r="I46" t="n">
         <v>0</v>
       </c>
@@ -10191,8 +10359,16 @@
           <t>5702427592-310-931003605894</t>
         </is>
       </c>
-      <c r="G51" t="inlineStr"/>
-      <c r="H51" t="inlineStr"/>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>وصف تفصيلي لـ SAPOFEN COLD &amp; FLU TABLET</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>SAPOFEN COLD &amp; FLU TABLET detailed description.</t>
+        </is>
+      </c>
       <c r="I51" t="n">
         <v>0</v>
       </c>
@@ -10374,8 +10550,16 @@
           <t>2471878945-560-804387619023</t>
         </is>
       </c>
-      <c r="G52" t="inlineStr"/>
-      <c r="H52" t="inlineStr"/>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>وصف تفصيلي لـ SAPOFEN 600 MG TAB</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>SAPOFEN 600 MG TAB detailed description.</t>
+        </is>
+      </c>
       <c r="I52" t="n">
         <v>0</v>
       </c>
@@ -10756,8 +10940,16 @@
           <t>9521578034-645-024314653778</t>
         </is>
       </c>
-      <c r="G54" t="inlineStr"/>
-      <c r="H54" t="inlineStr"/>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>وصف تفصيلي لـ SANSILLA GARGLE</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>SANSILLA GARGLE detailed description.</t>
+        </is>
+      </c>
       <c r="I54" t="n">
         <v>0</v>
       </c>
@@ -12937,8 +13129,16 @@
           <t>3219289482-785-512587486686</t>
         </is>
       </c>
-      <c r="G65" t="inlineStr"/>
-      <c r="H65" t="inlineStr"/>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>وصف تفصيلي لـ SECNEZOLE 500MG TABLETS</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>SECNEZOLE 500MG TABLETS detailed description.</t>
+        </is>
+      </c>
       <c r="I65" t="n">
         <v>0</v>
       </c>
@@ -13128,8 +13328,16 @@
           <t>1098728399-620-012615066015</t>
         </is>
       </c>
-      <c r="G66" t="inlineStr"/>
-      <c r="H66" t="inlineStr"/>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>وصف تفصيلي لـ SCANDICAINE 3% CARTRIDGE 1.8ML</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>SCANDICAINE 3% CARTRIDGE 1.8ML detailed description.</t>
+        </is>
+      </c>
       <c r="I66" t="n">
         <v>0</v>
       </c>
@@ -13323,8 +13531,16 @@
           <t>6933810200-703-208412605618</t>
         </is>
       </c>
-      <c r="G67" t="inlineStr"/>
-      <c r="H67" t="inlineStr"/>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>وصف تفصيلي لـ SCANDICAINE 2% SPECIALE CARTRIDGE</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>SCANDICAINE 2% SPECIALE CARTRIDGE detailed description.</t>
+        </is>
+      </c>
       <c r="I67" t="n">
         <v>0</v>
       </c>
@@ -13518,8 +13734,16 @@
           <t>7565982440-742-256949327903</t>
         </is>
       </c>
-      <c r="G68" t="inlineStr"/>
-      <c r="H68" t="inlineStr"/>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>وصف تفصيلي لـ SAXID 4MG TABLET</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>SAXID 4MG TABLET detailed description.</t>
+        </is>
+      </c>
       <c r="I68" t="n">
         <v>0</v>
       </c>
@@ -13705,8 +13929,16 @@
           <t>3778794845-805-950621848861</t>
         </is>
       </c>
-      <c r="G69" t="inlineStr"/>
-      <c r="H69" t="inlineStr"/>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>وصف تفصيلي لـ SAXID 2MG TABLET</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>SAXID 2MG TABLET detailed description.</t>
+        </is>
+      </c>
       <c r="I69" t="n">
         <v>0</v>
       </c>
@@ -13892,8 +14124,16 @@
           <t>0760281931-479-678220670345</t>
         </is>
       </c>
-      <c r="G70" t="inlineStr"/>
-      <c r="H70" t="inlineStr"/>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>وصف تفصيلي لـ SEDACID 20 MG COATED TABLETS</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>SEDACID 20 MG COATED TABLETS detailed description.</t>
+        </is>
+      </c>
       <c r="I70" t="n">
         <v>0</v>
       </c>
@@ -14871,8 +15111,16 @@
           <t>1289827161-347-821471681476</t>
         </is>
       </c>
-      <c r="G75" t="inlineStr"/>
-      <c r="H75" t="inlineStr"/>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>وصف تفصيلي لـ ROTATEQ ORAL VACCINE</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>ROTATEQ ORAL VACCINE detailed description.</t>
+        </is>
+      </c>
       <c r="I75" t="n">
         <v>0</v>
       </c>
@@ -16055,8 +16303,16 @@
           <t>3743494488-359-983672098955</t>
         </is>
       </c>
-      <c r="G81" t="inlineStr"/>
-      <c r="H81" t="inlineStr"/>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>وصف تفصيلي لـ SALIDEX TOPICAL SOLUTION</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>SALIDEX TOPICAL SOLUTION detailed description.</t>
+        </is>
+      </c>
       <c r="I81" t="n">
         <v>0</v>
       </c>
@@ -16242,8 +16498,16 @@
           <t>1717311934-424-530065081882</t>
         </is>
       </c>
-      <c r="G82" t="inlineStr"/>
-      <c r="H82" t="inlineStr"/>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>وصف تفصيلي لـ SALIDEX OINTMENT</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>SALIDEX OINTMENT detailed description.</t>
+        </is>
+      </c>
       <c r="I82" t="n">
         <v>0</v>
       </c>
@@ -16628,8 +16892,16 @@
           <t>3972328428-763-795870322989</t>
         </is>
       </c>
-      <c r="G84" t="inlineStr"/>
-      <c r="H84" t="inlineStr"/>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>وصف تفصيلي لـ RYTHINATE SUSP. 200MG-5ML</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>RYTHINATE SUSP. 200MG-5ML detailed description.</t>
+        </is>
+      </c>
       <c r="I84" t="n">
         <v>0</v>
       </c>
@@ -16819,8 +17091,16 @@
           <t>2035093348-633-412298775738</t>
         </is>
       </c>
-      <c r="G85" t="inlineStr"/>
-      <c r="H85" t="inlineStr"/>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>وصف تفصيلي لـ RUMAFEN</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>RUMAFEN detailed description.</t>
+        </is>
+      </c>
       <c r="I85" t="n">
         <v>0</v>
       </c>
@@ -17213,8 +17493,16 @@
           <t>1807980091-203-350039568573</t>
         </is>
       </c>
-      <c r="G87" t="inlineStr"/>
-      <c r="H87" t="inlineStr"/>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>وصف تفصيلي لـ SELEKTINE</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>SELEKTINE detailed description.</t>
+        </is>
+      </c>
       <c r="I87" t="n">
         <v>0</v>
       </c>
@@ -19350,8 +19638,16 @@
           <t>1304129472-839-070794358935</t>
         </is>
       </c>
-      <c r="G98" t="inlineStr"/>
-      <c r="H98" t="inlineStr"/>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>وصف تفصيلي لـ REPADERM GEL</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>REPADERM GEL detailed description.</t>
+        </is>
+      </c>
       <c r="I98" t="n">
         <v>0</v>
       </c>

</xml_diff>